<commit_message>
chore: Version 0.12.6.3 – LLM configs, relevance analyzer, response handling updates
</commit_message>
<xml_diff>
--- a/QCA-AID-Codebook.xlsx
+++ b/QCA-AID-Codebook.xlsx
@@ -1071,7 +1071,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Verfügbarkeit und Verteilung</t>
+          <t>verfügbarkeit und Verteilung</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1587,7 +1587,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>qwen2.5-coder:7b</t>
+          <t>qwen/qwen3.6-35b-a3b</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -1631,7 +1631,7 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="E6" t="inlineStr"/>
     </row>
@@ -1710,7 +1710,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>deductive</t>
+          <t>abductive</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1895,6 +1895,43 @@
       </c>
       <c r="E22" t="inlineStr"/>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>relevance_threshold</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>enable_optimization</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>api_base_url</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>